<commit_message>
feat: verify rule CG0087 and add negative test cases
</commit_message>
<xml_diff>
--- a/rules/CORE-000014/negative/01/data/unit-test-coreid-CG0087-negative.xlsx
+++ b/rules/CORE-000014/negative/01/data/unit-test-coreid-CG0087-negative.xlsx
@@ -1,29 +1,29 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Library" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Datasets" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Validation" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="ag.xpt" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="cm.xpt" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="ec.xpt" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="ex.xpt" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="ml.xpt" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="pr.xpt" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="su.xpt" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="ae.xpt" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="be.xpt" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="ce.xpt" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="ds.xpt" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="dv.xpt" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="ho.xpt" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="mh.xpt" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Library" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Datasets" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Validation" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ag.xpt" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cm.xpt" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ec.xpt" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ex.xpt" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ml.xpt" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pr.xpt" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="su.xpt" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ae.xpt" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="be.xpt" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ce.xpt" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ds.xpt" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="dv.xpt" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ho.xpt" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="mh.xpt" sheetId="17" state="visible" r:id="rId17"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -48,7 +48,7 @@
       <i val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -59,6 +59,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00FFFFCC"/>
         <bgColor rgb="00FFFFCC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor rgb="FFFFFF00"/>
       </patternFill>
     </fill>
   </fills>
@@ -104,7 +110,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -124,6 +130,10 @@
     </xf>
     <xf numFmtId="49" fontId="2" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -707,11 +717,13 @@
           <t>CIGARETTES</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="F5" s="8" t="n"/>
+      <c r="G5" s="9" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
+      <c r="H5" s="8" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -737,12 +749,13 @@
           <t>CAFFEINE</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="F6" s="8" t="n"/>
+      <c r="G6" s="9" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="H6" s="9" t="inlineStr">
         <is>
           <t>NOT DONE</t>
         </is>
@@ -772,11 +785,13 @@
           <t>TOBACCO</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="F7" s="8" t="n"/>
+      <c r="G7" s="9" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
+      <c r="H7" s="8" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1176,13 +1191,13 @@
           <t>Collecting</t>
         </is>
       </c>
-      <c r="F5" s="5" t="n"/>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="F5" s="9" t="n"/>
+      <c r="G5" s="9" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="H5" s="5" t="n"/>
+      <c r="H5" s="9" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -1208,13 +1223,13 @@
           <t>Extracting</t>
         </is>
       </c>
-      <c r="F6" s="5" t="n"/>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="F6" s="9" t="n"/>
+      <c r="G6" s="9" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H6" s="5" t="n"/>
+      <c r="H6" s="9" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -1240,13 +1255,13 @@
           <t>Shipping</t>
         </is>
       </c>
-      <c r="F7" s="5" t="n"/>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="F7" s="9" t="n"/>
+      <c r="G7" s="9" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="H7" s="9" t="inlineStr">
         <is>
           <t>NOT DONE</t>
         </is>
@@ -1276,13 +1291,13 @@
           <t>Aliquoting</t>
         </is>
       </c>
-      <c r="F8" s="5" t="n"/>
-      <c r="G8" s="5" t="inlineStr">
+      <c r="F8" s="9" t="n"/>
+      <c r="G8" s="9" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H8" s="5" t="n"/>
+      <c r="H8" s="9" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1474,11 +1489,13 @@
           <t>Rash</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="F5" s="8" t="n"/>
+      <c r="G5" s="9" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
+      <c r="H5" s="8" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -1504,11 +1521,13 @@
           <t>Wheezing</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="F6" s="8" t="n"/>
+      <c r="G6" s="9" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H6" s="8" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -1534,12 +1553,13 @@
           <t>Edema</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="F7" s="8" t="n"/>
+      <c r="G7" s="9" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="H7" s="9" t="inlineStr">
         <is>
           <t>NOT DONE</t>
         </is>
@@ -1569,11 +1589,13 @@
           <t>Conjunctivitis</t>
         </is>
       </c>
-      <c r="G8" s="5" t="inlineStr">
+      <c r="F8" s="8" t="n"/>
+      <c r="G8" s="9" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H8" s="8" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2335,11 +2357,13 @@
           <t>HOSPITAL</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="F5" s="8" t="n"/>
+      <c r="G5" s="9" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
+      <c r="H5" s="8" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -2365,11 +2389,13 @@
           <t>NURSING HOME</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="F6" s="8" t="n"/>
+      <c r="G6" s="9" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H6" s="8" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -2395,12 +2421,13 @@
           <t>GENERAL WARD</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="F7" s="8" t="n"/>
+      <c r="G7" s="9" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="H7" s="9" t="inlineStr">
         <is>
           <t>NOT DONE</t>
         </is>
@@ -2430,11 +2457,13 @@
           <t>INTENSIVE CARE</t>
         </is>
       </c>
-      <c r="G8" s="5" t="inlineStr">
+      <c r="F8" s="8" t="n"/>
+      <c r="G8" s="9" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H8" s="8" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2626,11 +2655,13 @@
           <t>ASTHMA</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="F5" s="8" t="n"/>
+      <c r="G5" s="9" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
+      <c r="H5" s="8" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -2656,12 +2687,13 @@
           <t>CONGESTIVE HEART FAILURE</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="F6" s="8" t="n"/>
+      <c r="G6" s="9" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="H6" s="9" t="inlineStr">
         <is>
           <t>NOT DONE</t>
         </is>
@@ -2691,12 +2723,13 @@
           <t>BROKEN LEG</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="F7" s="8" t="n"/>
+      <c r="G7" s="9" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="H7" s="9" t="inlineStr">
         <is>
           <t>NOT DONE</t>
         </is>
@@ -2726,11 +2759,13 @@
           <t>HEADACHES</t>
         </is>
       </c>
-      <c r="G8" s="5" t="inlineStr">
+      <c r="F8" s="8" t="n"/>
+      <c r="G8" s="9" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H8" s="8" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2937,7 +2972,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2969,6 +3004,2587 @@
       <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Error value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ag.xpt</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>5</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>AGOCCUR</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>ag.xpt</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>5</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>AGPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>ag.xpt</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>5</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>AGSTAT</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ag.xpt</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>6</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>AGOCCUR</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ag.xpt</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>6</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>AGPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ag.xpt</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>6</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>AGSTAT</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>3</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>ag.xpt</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>7</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>AGOCCUR</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>3</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>ag.xpt</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>7</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>AGPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>3</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>ag.xpt</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>7</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>AGSTAT</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>NOT DONE</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>4</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>cm.xpt</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>5</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>CMOCCUR</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>4</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>cm.xpt</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>5</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>CMPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>4</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>cm.xpt</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>5</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>CMSTAT</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>5</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>cm.xpt</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>6</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>CMOCCUR</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>5</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>cm.xpt</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>6</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>CMPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>5</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>cm.xpt</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>6</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>CMSTAT</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>6</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>cm.xpt</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>7</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>CMOCCUR</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>6</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>cm.xpt</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>7</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>CMPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>6</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>cm.xpt</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>7</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>CMSTAT</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>NOT DONE</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>7</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>ec.xpt</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>5</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>ECOCCUR</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>7</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>ec.xpt</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>5</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>ECPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>7</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>ec.xpt</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>5</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>ECSTAT</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Not in dataset</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>8</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>ec.xpt</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>6</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>ECOCCUR</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>8</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>ec.xpt</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>6</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>ECPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>8</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>ec.xpt</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>6</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>ECSTAT</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Not in dataset</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>9</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>ec.xpt</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>7</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>ECOCCUR</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>9</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>ec.xpt</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>7</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>ECPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>9</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>ec.xpt</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>7</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>ECSTAT</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Not in dataset</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>10</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>ml.xpt</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>5</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>MLOCCUR</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>10</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>ml.xpt</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>5</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>MLPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>10</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>ml.xpt</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>5</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>MLSTAT</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>11</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>ml.xpt</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>6</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>MLOCCUR</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>11</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>ml.xpt</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>6</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>MLPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>11</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>ml.xpt</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>6</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>MLSTAT</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>12</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>ml.xpt</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>7</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>MLOCCUR</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>12</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>ml.xpt</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>7</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>MLPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>12</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>ml.xpt</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>7</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>MLSTAT</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>NOT DONE</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>13</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>pr.xpt</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>5</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>PROCCUR</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>13</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>pr.xpt</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>5</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>PRPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>13</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>pr.xpt</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>5</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>PRSTAT</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>14</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>pr.xpt</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>6</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>PROCCUR</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>14</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>pr.xpt</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>6</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>PRPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>14</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>pr.xpt</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>6</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>PRSTAT</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>NOT DONE</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>15</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>pr.xpt</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>7</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>PROCCUR</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>15</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>pr.xpt</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>7</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>PRPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>15</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>pr.xpt</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>7</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>PRSTAT</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>16</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>su.xpt</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>5</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>SUOCCUR</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>16</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>su.xpt</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>5</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>SUPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>16</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>su.xpt</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>5</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>SUSTAT</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>17</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>su.xpt</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>6</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>SUOCCUR</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>17</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>su.xpt</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>6</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>SUPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>17</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>su.xpt</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>6</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>SUSTAT</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>NOT DONE</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>18</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>su.xpt</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>7</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>SUOCCUR</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>18</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>su.xpt</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>7</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>SUPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>18</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>su.xpt</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>7</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>SUSTAT</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>19</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>be.xpt</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>5</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>BEOCCUR</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>19</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>be.xpt</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>5</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>BEPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>19</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>be.xpt</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>5</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>BESTAT</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>20</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>be.xpt</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>6</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>BEOCCUR</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>20</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>be.xpt</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>6</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>BEPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>20</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>be.xpt</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>6</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>BESTAT</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>21</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>be.xpt</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>7</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>BEOCCUR</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
+        <v>21</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>be.xpt</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>7</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>BEPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
+        <v>21</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>be.xpt</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>7</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>BESTAT</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>NOT DONE</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="n">
+        <v>22</v>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>be.xpt</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>8</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>BEOCCUR</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="n">
+        <v>22</v>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>be.xpt</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>8</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>BEPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="n">
+        <v>22</v>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>be.xpt</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>8</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>BESTAT</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="n">
+        <v>23</v>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>ce.xpt</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>5</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>CEOCCUR</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="n">
+        <v>23</v>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>ce.xpt</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>5</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>CEPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="n">
+        <v>23</v>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>ce.xpt</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>5</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>CESTAT</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="n">
+        <v>24</v>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>ce.xpt</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>6</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>CEOCCUR</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="n">
+        <v>24</v>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>ce.xpt</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
+        <v>6</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>CEPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="n">
+        <v>24</v>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>ce.xpt</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D73" t="n">
+        <v>6</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>CESTAT</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="n">
+        <v>25</v>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>ce.xpt</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D74" t="n">
+        <v>7</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>CEOCCUR</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="n">
+        <v>25</v>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>ce.xpt</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D75" t="n">
+        <v>7</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>CEPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="n">
+        <v>25</v>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>ce.xpt</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D76" t="n">
+        <v>7</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>CESTAT</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>NOT DONE</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="n">
+        <v>26</v>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>ce.xpt</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
+        <v>8</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>CEOCCUR</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="n">
+        <v>26</v>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>ce.xpt</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D78" t="n">
+        <v>8</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>CEPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="n">
+        <v>26</v>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>ce.xpt</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D79" t="n">
+        <v>8</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>CESTAT</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="n">
+        <v>27</v>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>ho.xpt</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D80" t="n">
+        <v>5</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>HOOCCUR</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="n">
+        <v>27</v>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>ho.xpt</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D81" t="n">
+        <v>5</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>HOPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="n">
+        <v>27</v>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>ho.xpt</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D82" t="n">
+        <v>5</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>HOSTAT</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="n">
+        <v>28</v>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>ho.xpt</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D83" t="n">
+        <v>6</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>HOOCCUR</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="n">
+        <v>28</v>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>ho.xpt</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D84" t="n">
+        <v>6</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>HOPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="n">
+        <v>28</v>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>ho.xpt</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D85" t="n">
+        <v>6</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>HOSTAT</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="n">
+        <v>29</v>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>ho.xpt</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D86" t="n">
+        <v>7</v>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>HOOCCUR</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="n">
+        <v>29</v>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>ho.xpt</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D87" t="n">
+        <v>7</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>HOPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="n">
+        <v>29</v>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>ho.xpt</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D88" t="n">
+        <v>7</v>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>HOSTAT</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>NOT DONE</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="n">
+        <v>30</v>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>ho.xpt</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D89" t="n">
+        <v>8</v>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>HOOCCUR</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="n">
+        <v>30</v>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>ho.xpt</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D90" t="n">
+        <v>8</v>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>HOPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="n">
+        <v>30</v>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>ho.xpt</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D91" t="n">
+        <v>8</v>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>HOSTAT</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="n">
+        <v>31</v>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>mh.xpt</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D92" t="n">
+        <v>5</v>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>MHOCCUR</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="n">
+        <v>31</v>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>mh.xpt</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D93" t="n">
+        <v>5</v>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>MHPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="n">
+        <v>31</v>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>mh.xpt</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D94" t="n">
+        <v>5</v>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>MHSTAT</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="n">
+        <v>32</v>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>mh.xpt</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D95" t="n">
+        <v>6</v>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>MHOCCUR</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="n">
+        <v>32</v>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>mh.xpt</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D96" t="n">
+        <v>6</v>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>MHPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="n">
+        <v>32</v>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>mh.xpt</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D97" t="n">
+        <v>6</v>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>MHSTAT</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>NOT DONE</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="n">
+        <v>33</v>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>mh.xpt</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D98" t="n">
+        <v>7</v>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>MHOCCUR</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="n">
+        <v>33</v>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>mh.xpt</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D99" t="n">
+        <v>7</v>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>MHPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="n">
+        <v>33</v>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>mh.xpt</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D100" t="n">
+        <v>7</v>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>MHSTAT</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>NOT DONE</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="n">
+        <v>34</v>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>mh.xpt</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D101" t="n">
+        <v>8</v>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>MHOCCUR</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="n">
+        <v>34</v>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>mh.xpt</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D102" t="n">
+        <v>8</v>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>MHPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="n">
+        <v>34</v>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>mh.xpt</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D103" t="n">
+        <v>8</v>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>MHSTAT</t>
         </is>
       </c>
     </row>
@@ -3162,11 +5778,13 @@
           <t>Buprenorphine</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="F5" s="8" t="n"/>
+      <c r="G5" s="9" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
+      <c r="H5" s="8" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -3192,11 +5810,13 @@
           <t>Minims Proxymetacaine</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="F6" s="8" t="n"/>
+      <c r="G6" s="9" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H6" s="8" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -3222,12 +5842,13 @@
           <t>Meloxicam</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="F7" s="8" t="n"/>
+      <c r="G7" s="9" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="H7" s="9" t="inlineStr">
         <is>
           <t>NOT DONE</t>
         </is>
@@ -3423,11 +6044,13 @@
           <t>ASPIRIN</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="F5" s="8" t="n"/>
+      <c r="G5" s="9" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
+      <c r="H5" s="8" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -3453,11 +6076,13 @@
           <t>METAMUCIL</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="F6" s="8" t="n"/>
+      <c r="G6" s="9" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H6" s="8" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -3483,12 +6108,13 @@
           <t>HYDROCORTISONE, TOPICAL</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="F7" s="8" t="n"/>
+      <c r="G7" s="9" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="H7" s="9" t="inlineStr">
         <is>
           <t>NOT DONE</t>
         </is>
@@ -3666,7 +6292,8 @@
           <t>ZANOMALINE</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="F5" s="8" t="n"/>
+      <c r="G5" s="9" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -3696,7 +6323,8 @@
           <t>ZANOMALINE</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="F6" s="8" t="n"/>
+      <c r="G6" s="9" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -3726,7 +6354,8 @@
           <t>ZANOMALINE</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="F7" s="8" t="n"/>
+      <c r="G7" s="9" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -4202,11 +6831,13 @@
           <t>SNACK</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="F5" s="8" t="n"/>
+      <c r="G5" s="9" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
+      <c r="H5" s="8" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -4232,11 +6863,13 @@
           <t>NUTRITIONAL DRINK</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="F6" s="8" t="n"/>
+      <c r="G6" s="9" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H6" s="8" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -4262,12 +6895,13 @@
           <t>WILD MUSHROOMS</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="F7" s="8" t="n"/>
+      <c r="G7" s="9" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="H7" s="9" t="inlineStr">
         <is>
           <t>NOT DONE</t>
         </is>
@@ -4463,12 +7097,13 @@
           <t>Wisdom Teeth Extraction</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="F5" s="8" t="n"/>
+      <c r="G5" s="9" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="H5" s="5" t="n"/>
+      <c r="H5" s="9" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -4494,12 +7129,13 @@
           <t>Endoscopy</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="F6" s="8" t="n"/>
+      <c r="G6" s="9" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="H6" s="9" t="inlineStr">
         <is>
           <t>NOT DONE</t>
         </is>
@@ -4529,12 +7165,13 @@
           <t>Heart Transplant</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="F7" s="8" t="n"/>
+      <c r="G7" s="9" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="H7" s="5" t="n"/>
+      <c r="H7" s="9" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
fix: highlight issues in the negative test case
</commit_message>
<xml_diff>
--- a/rules/CORE-000014/negative/01/data/unit-test-coreid-CG0087-negative.xlsx
+++ b/rules/CORE-000014/negative/01/data/unit-test-coreid-CG0087-negative.xlsx
@@ -1,29 +1,29 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Library" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Datasets" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Validation" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ag.xpt" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cm.xpt" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ec.xpt" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ex.xpt" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ml.xpt" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pr.xpt" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="su.xpt" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ae.xpt" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="be.xpt" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ce.xpt" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ds.xpt" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="dv.xpt" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ho.xpt" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="mh.xpt" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="Library" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Datasets" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Validation" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="ag.xpt" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="cm.xpt" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="ec.xpt" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="ex.xpt" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="ml.xpt" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="pr.xpt" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="su.xpt" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="ae.xpt" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="be.xpt" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="ce.xpt" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="ds.xpt" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="dv.xpt" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="ho.xpt" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="mh.xpt" sheetId="17" state="visible" r:id="rId17"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3536,7 +3536,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Not in dataset</t>
+          <t>[ABSENT]</t>
         </is>
       </c>
     </row>
@@ -3615,7 +3615,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Not in dataset</t>
+          <t>[ABSENT]</t>
         </is>
       </c>
     </row>
@@ -3694,7 +3694,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Not in dataset</t>
+          <t>[ABSENT]</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
restore conflicting core ids
</commit_message>
<xml_diff>
--- a/rules/CORE-000014/negative/01/data/unit-test-coreid-CG0087-negative.xlsx
+++ b/rules/CORE-000014/negative/01/data/unit-test-coreid-CG0087-negative.xlsx
@@ -48,7 +48,7 @@
       <i val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -59,6 +59,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00FFFFCC"/>
         <bgColor rgb="00FFFFCC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor rgb="FFFFFF00"/>
       </patternFill>
     </fill>
   </fills>
@@ -104,7 +110,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -124,6 +130,10 @@
     </xf>
     <xf numFmtId="49" fontId="2" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -707,11 +717,13 @@
           <t>CIGARETTES</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="F5" s="8" t="n"/>
+      <c r="G5" s="9" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
+      <c r="H5" s="8" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -737,12 +749,13 @@
           <t>CAFFEINE</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="F6" s="8" t="n"/>
+      <c r="G6" s="9" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="H6" s="9" t="inlineStr">
         <is>
           <t>NOT DONE</t>
         </is>
@@ -772,11 +785,13 @@
           <t>TOBACCO</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="F7" s="8" t="n"/>
+      <c r="G7" s="9" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
+      <c r="H7" s="8" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1176,13 +1191,13 @@
           <t>Collecting</t>
         </is>
       </c>
-      <c r="F5" s="5" t="n"/>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="F5" s="9" t="n"/>
+      <c r="G5" s="9" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="H5" s="5" t="n"/>
+      <c r="H5" s="9" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -1208,13 +1223,13 @@
           <t>Extracting</t>
         </is>
       </c>
-      <c r="F6" s="5" t="n"/>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="F6" s="9" t="n"/>
+      <c r="G6" s="9" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H6" s="5" t="n"/>
+      <c r="H6" s="9" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -1240,13 +1255,13 @@
           <t>Shipping</t>
         </is>
       </c>
-      <c r="F7" s="5" t="n"/>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="F7" s="9" t="n"/>
+      <c r="G7" s="9" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="H7" s="9" t="inlineStr">
         <is>
           <t>NOT DONE</t>
         </is>
@@ -1276,13 +1291,13 @@
           <t>Aliquoting</t>
         </is>
       </c>
-      <c r="F8" s="5" t="n"/>
-      <c r="G8" s="5" t="inlineStr">
+      <c r="F8" s="9" t="n"/>
+      <c r="G8" s="9" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H8" s="5" t="n"/>
+      <c r="H8" s="9" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1474,11 +1489,13 @@
           <t>Rash</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="F5" s="8" t="n"/>
+      <c r="G5" s="9" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
+      <c r="H5" s="8" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -1504,11 +1521,13 @@
           <t>Wheezing</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="F6" s="8" t="n"/>
+      <c r="G6" s="9" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H6" s="8" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -1534,12 +1553,13 @@
           <t>Edema</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="F7" s="8" t="n"/>
+      <c r="G7" s="9" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="H7" s="9" t="inlineStr">
         <is>
           <t>NOT DONE</t>
         </is>
@@ -1569,11 +1589,13 @@
           <t>Conjunctivitis</t>
         </is>
       </c>
-      <c r="G8" s="5" t="inlineStr">
+      <c r="F8" s="8" t="n"/>
+      <c r="G8" s="9" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H8" s="8" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2335,11 +2357,13 @@
           <t>HOSPITAL</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="F5" s="8" t="n"/>
+      <c r="G5" s="9" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
+      <c r="H5" s="8" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -2365,11 +2389,13 @@
           <t>NURSING HOME</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="F6" s="8" t="n"/>
+      <c r="G6" s="9" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H6" s="8" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -2395,12 +2421,13 @@
           <t>GENERAL WARD</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="F7" s="8" t="n"/>
+      <c r="G7" s="9" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="H7" s="9" t="inlineStr">
         <is>
           <t>NOT DONE</t>
         </is>
@@ -2430,11 +2457,13 @@
           <t>INTENSIVE CARE</t>
         </is>
       </c>
-      <c r="G8" s="5" t="inlineStr">
+      <c r="F8" s="8" t="n"/>
+      <c r="G8" s="9" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H8" s="8" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2626,11 +2655,13 @@
           <t>ASTHMA</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="F5" s="8" t="n"/>
+      <c r="G5" s="9" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
+      <c r="H5" s="8" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -2656,12 +2687,13 @@
           <t>CONGESTIVE HEART FAILURE</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="F6" s="8" t="n"/>
+      <c r="G6" s="9" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="H6" s="9" t="inlineStr">
         <is>
           <t>NOT DONE</t>
         </is>
@@ -2691,12 +2723,13 @@
           <t>BROKEN LEG</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="F7" s="8" t="n"/>
+      <c r="G7" s="9" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="H7" s="9" t="inlineStr">
         <is>
           <t>NOT DONE</t>
         </is>
@@ -2726,11 +2759,13 @@
           <t>HEADACHES</t>
         </is>
       </c>
-      <c r="G8" s="5" t="inlineStr">
+      <c r="F8" s="8" t="n"/>
+      <c r="G8" s="9" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H8" s="8" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2937,7 +2972,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2969,6 +3004,2587 @@
       <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Error value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ag.xpt</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>5</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>AGOCCUR</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>ag.xpt</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>5</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>AGPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>ag.xpt</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>5</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>AGSTAT</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ag.xpt</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>6</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>AGOCCUR</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ag.xpt</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>6</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>AGPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ag.xpt</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>6</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>AGSTAT</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>3</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>ag.xpt</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>7</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>AGOCCUR</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>3</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>ag.xpt</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>7</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>AGPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>3</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>ag.xpt</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>7</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>AGSTAT</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>NOT DONE</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>4</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>cm.xpt</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>5</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>CMOCCUR</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>4</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>cm.xpt</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>5</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>CMPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>4</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>cm.xpt</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>5</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>CMSTAT</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>5</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>cm.xpt</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>6</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>CMOCCUR</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>5</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>cm.xpt</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>6</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>CMPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>5</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>cm.xpt</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>6</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>CMSTAT</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>6</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>cm.xpt</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>7</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>CMOCCUR</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>6</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>cm.xpt</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>7</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>CMPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>6</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>cm.xpt</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>7</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>CMSTAT</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>NOT DONE</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>7</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>ec.xpt</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>5</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>ECOCCUR</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>7</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>ec.xpt</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>5</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>ECPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>7</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>ec.xpt</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>5</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>ECSTAT</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>[ABSENT]</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>8</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>ec.xpt</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>6</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>ECOCCUR</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>8</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>ec.xpt</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>6</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>ECPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>8</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>ec.xpt</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>6</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>ECSTAT</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>[ABSENT]</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>9</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>ec.xpt</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>7</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>ECOCCUR</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>9</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>ec.xpt</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>7</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>ECPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>9</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>ec.xpt</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>7</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>ECSTAT</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>[ABSENT]</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>10</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>ml.xpt</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>5</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>MLOCCUR</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>10</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>ml.xpt</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>5</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>MLPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>10</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>ml.xpt</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>5</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>MLSTAT</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>11</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>ml.xpt</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>6</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>MLOCCUR</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>11</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>ml.xpt</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>6</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>MLPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>11</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>ml.xpt</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>6</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>MLSTAT</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>12</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>ml.xpt</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>7</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>MLOCCUR</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>12</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>ml.xpt</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>7</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>MLPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>12</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>ml.xpt</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>7</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>MLSTAT</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>NOT DONE</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>13</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>pr.xpt</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>5</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>PROCCUR</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>13</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>pr.xpt</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>5</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>PRPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>13</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>pr.xpt</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>5</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>PRSTAT</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>14</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>pr.xpt</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>6</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>PROCCUR</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>14</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>pr.xpt</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>6</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>PRPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>14</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>pr.xpt</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>6</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>PRSTAT</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>NOT DONE</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>15</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>pr.xpt</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>7</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>PROCCUR</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>15</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>pr.xpt</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>7</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>PRPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>15</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>pr.xpt</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>7</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>PRSTAT</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>16</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>su.xpt</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>5</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>SUOCCUR</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>16</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>su.xpt</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>5</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>SUPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>16</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>su.xpt</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>5</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>SUSTAT</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>17</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>su.xpt</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>6</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>SUOCCUR</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>17</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>su.xpt</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>6</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>SUPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>17</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>su.xpt</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>6</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>SUSTAT</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>NOT DONE</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>18</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>su.xpt</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>7</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>SUOCCUR</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>18</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>su.xpt</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>7</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>SUPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>18</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>su.xpt</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>7</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>SUSTAT</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>19</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>be.xpt</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>5</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>BEOCCUR</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>19</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>be.xpt</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>5</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>BEPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>19</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>be.xpt</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>5</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>BESTAT</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>20</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>be.xpt</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>6</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>BEOCCUR</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>20</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>be.xpt</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>6</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>BEPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>20</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>be.xpt</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>6</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>BESTAT</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>21</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>be.xpt</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>7</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>BEOCCUR</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
+        <v>21</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>be.xpt</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>7</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>BEPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
+        <v>21</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>be.xpt</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>7</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>BESTAT</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>NOT DONE</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="n">
+        <v>22</v>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>be.xpt</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>8</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>BEOCCUR</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="n">
+        <v>22</v>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>be.xpt</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>8</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>BEPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="n">
+        <v>22</v>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>be.xpt</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>8</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>BESTAT</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="n">
+        <v>23</v>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>ce.xpt</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>5</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>CEOCCUR</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="n">
+        <v>23</v>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>ce.xpt</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>5</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>CEPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="n">
+        <v>23</v>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>ce.xpt</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>5</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>CESTAT</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="n">
+        <v>24</v>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>ce.xpt</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>6</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>CEOCCUR</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="n">
+        <v>24</v>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>ce.xpt</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
+        <v>6</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>CEPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="n">
+        <v>24</v>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>ce.xpt</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D73" t="n">
+        <v>6</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>CESTAT</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="n">
+        <v>25</v>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>ce.xpt</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D74" t="n">
+        <v>7</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>CEOCCUR</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="n">
+        <v>25</v>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>ce.xpt</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D75" t="n">
+        <v>7</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>CEPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="n">
+        <v>25</v>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>ce.xpt</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D76" t="n">
+        <v>7</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>CESTAT</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>NOT DONE</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="n">
+        <v>26</v>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>ce.xpt</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
+        <v>8</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>CEOCCUR</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="n">
+        <v>26</v>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>ce.xpt</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D78" t="n">
+        <v>8</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>CEPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="n">
+        <v>26</v>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>ce.xpt</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D79" t="n">
+        <v>8</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>CESTAT</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="n">
+        <v>27</v>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>ho.xpt</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D80" t="n">
+        <v>5</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>HOOCCUR</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="n">
+        <v>27</v>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>ho.xpt</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D81" t="n">
+        <v>5</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>HOPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="n">
+        <v>27</v>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>ho.xpt</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D82" t="n">
+        <v>5</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>HOSTAT</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="n">
+        <v>28</v>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>ho.xpt</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D83" t="n">
+        <v>6</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>HOOCCUR</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="n">
+        <v>28</v>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>ho.xpt</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D84" t="n">
+        <v>6</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>HOPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="n">
+        <v>28</v>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>ho.xpt</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D85" t="n">
+        <v>6</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>HOSTAT</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="n">
+        <v>29</v>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>ho.xpt</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D86" t="n">
+        <v>7</v>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>HOOCCUR</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="n">
+        <v>29</v>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>ho.xpt</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D87" t="n">
+        <v>7</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>HOPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="n">
+        <v>29</v>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>ho.xpt</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D88" t="n">
+        <v>7</v>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>HOSTAT</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>NOT DONE</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="n">
+        <v>30</v>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>ho.xpt</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D89" t="n">
+        <v>8</v>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>HOOCCUR</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="n">
+        <v>30</v>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>ho.xpt</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D90" t="n">
+        <v>8</v>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>HOPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="n">
+        <v>30</v>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>ho.xpt</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D91" t="n">
+        <v>8</v>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>HOSTAT</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="n">
+        <v>31</v>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>mh.xpt</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D92" t="n">
+        <v>5</v>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>MHOCCUR</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="n">
+        <v>31</v>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>mh.xpt</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D93" t="n">
+        <v>5</v>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>MHPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="n">
+        <v>31</v>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>mh.xpt</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D94" t="n">
+        <v>5</v>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>MHSTAT</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="n">
+        <v>32</v>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>mh.xpt</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D95" t="n">
+        <v>6</v>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>MHOCCUR</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="n">
+        <v>32</v>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>mh.xpt</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D96" t="n">
+        <v>6</v>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>MHPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="n">
+        <v>32</v>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>mh.xpt</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D97" t="n">
+        <v>6</v>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>MHSTAT</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>NOT DONE</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="n">
+        <v>33</v>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>mh.xpt</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D98" t="n">
+        <v>7</v>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>MHOCCUR</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="n">
+        <v>33</v>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>mh.xpt</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D99" t="n">
+        <v>7</v>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>MHPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="n">
+        <v>33</v>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>mh.xpt</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D100" t="n">
+        <v>7</v>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>MHSTAT</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>NOT DONE</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="n">
+        <v>34</v>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>mh.xpt</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D101" t="n">
+        <v>8</v>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>MHOCCUR</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="n">
+        <v>34</v>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>mh.xpt</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D102" t="n">
+        <v>8</v>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>MHPRESP</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="n">
+        <v>34</v>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>mh.xpt</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D103" t="n">
+        <v>8</v>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>MHSTAT</t>
         </is>
       </c>
     </row>
@@ -3162,11 +5778,13 @@
           <t>Buprenorphine</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="F5" s="8" t="n"/>
+      <c r="G5" s="9" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
+      <c r="H5" s="8" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -3192,11 +5810,13 @@
           <t>Minims Proxymetacaine</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="F6" s="8" t="n"/>
+      <c r="G6" s="9" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H6" s="8" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -3222,12 +5842,13 @@
           <t>Meloxicam</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="F7" s="8" t="n"/>
+      <c r="G7" s="9" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="H7" s="9" t="inlineStr">
         <is>
           <t>NOT DONE</t>
         </is>
@@ -3423,11 +6044,13 @@
           <t>ASPIRIN</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="F5" s="8" t="n"/>
+      <c r="G5" s="9" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
+      <c r="H5" s="8" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -3453,11 +6076,13 @@
           <t>METAMUCIL</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="F6" s="8" t="n"/>
+      <c r="G6" s="9" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H6" s="8" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -3483,12 +6108,13 @@
           <t>HYDROCORTISONE, TOPICAL</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="F7" s="8" t="n"/>
+      <c r="G7" s="9" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="H7" s="9" t="inlineStr">
         <is>
           <t>NOT DONE</t>
         </is>
@@ -3666,7 +6292,8 @@
           <t>ZANOMALINE</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="F5" s="8" t="n"/>
+      <c r="G5" s="9" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -3696,7 +6323,8 @@
           <t>ZANOMALINE</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="F6" s="8" t="n"/>
+      <c r="G6" s="9" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -3726,7 +6354,8 @@
           <t>ZANOMALINE</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="F7" s="8" t="n"/>
+      <c r="G7" s="9" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -4202,11 +6831,13 @@
           <t>SNACK</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="F5" s="8" t="n"/>
+      <c r="G5" s="9" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
+      <c r="H5" s="8" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -4232,11 +6863,13 @@
           <t>NUTRITIONAL DRINK</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="F6" s="8" t="n"/>
+      <c r="G6" s="9" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H6" s="8" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -4262,12 +6895,13 @@
           <t>WILD MUSHROOMS</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="F7" s="8" t="n"/>
+      <c r="G7" s="9" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="H7" s="9" t="inlineStr">
         <is>
           <t>NOT DONE</t>
         </is>
@@ -4463,12 +7097,13 @@
           <t>Wisdom Teeth Extraction</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="F5" s="8" t="n"/>
+      <c r="G5" s="9" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="H5" s="5" t="n"/>
+      <c r="H5" s="9" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -4494,12 +7129,13 @@
           <t>Endoscopy</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="F6" s="8" t="n"/>
+      <c r="G6" s="9" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="H6" s="9" t="inlineStr">
         <is>
           <t>NOT DONE</t>
         </is>
@@ -4529,12 +7165,13 @@
           <t>Heart Transplant</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="F7" s="8" t="n"/>
+      <c r="G7" s="9" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="H7" s="5" t="n"/>
+      <c r="H7" s="9" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>